<commit_message>
feat: support first sheet index upload and reading for benefits and tax workbooks
</commit_message>
<xml_diff>
--- a/data/benefits.xlsx
+++ b/data/benefits.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Data" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="MyCustomSheet" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -22,7 +22,7 @@
     <t>Batch Arguments/JVM Arguments</t>
   </si>
   <si>
-    <t>TestDataBatch</t>
+    <t>TestCustomSheetBatch</t>
   </si>
   <si>
     <t>benefits_daily_6am</t>

</xml_diff>

<commit_message>
fix(upload): harden excel parsing to always read sheet index 0 with flexible header matching
</commit_message>
<xml_diff>
--- a/data/benefits.xlsx
+++ b/data/benefits.xlsx
@@ -4,31 +4,37 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="MyCustomSheet" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
-  <si>
-    <t>Batch Name/Job Name</t>
-  </si>
-  <si>
-    <t>Schedule Name/ Job Group Name</t>
-  </si>
-  <si>
-    <t>Batch Arguments/JVM Arguments</t>
-  </si>
-  <si>
-    <t>TestCustomSheetBatch</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+  <si>
+    <t>Job</t>
+  </si>
+  <si>
+    <t>Args</t>
+  </si>
+  <si>
+    <t>Schedule</t>
+  </si>
+  <si>
+    <t>Trigger</t>
+  </si>
+  <si>
+    <t>CustomHeaderBatch</t>
+  </si>
+  <si>
+    <t>-Denv=test</t>
   </si>
   <si>
     <t>benefits_daily_6am</t>
   </si>
   <si>
-    <t>-Xmx512m</t>
+    <t>Y</t>
   </si>
 </sst>
 </file>
@@ -405,10 +411,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -418,16 +424,22 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="D2" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: ensure persistent storage and automatic retention of uploaded benefits and tax sheets
</commit_message>
<xml_diff>
--- a/data/benefits.xlsx
+++ b/data/benefits.xlsx
@@ -4,44 +4,215 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="Benefits" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
-  <si>
-    <t>Job</t>
-  </si>
-  <si>
-    <t>Args</t>
-  </si>
-  <si>
-    <t>Schedule</t>
-  </si>
-  <si>
-    <t>Trigger</t>
-  </si>
-  <si>
-    <t>CustomHeaderBatch</t>
-  </si>
-  <si>
-    <t>-Denv=test</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="65">
+  <si>
+    <t>Batch Name/Job Name</t>
+  </si>
+  <si>
+    <t>Batch Arguments/JVM Arguments</t>
+  </si>
+  <si>
+    <t>Schedule Name/ Job Group Name</t>
+  </si>
+  <si>
+    <t>Trigger Needed</t>
+  </si>
+  <si>
+    <t>BatchEnrollmentSync</t>
+  </si>
+  <si>
+    <t>ENV=PROD,TENANT=benefits</t>
   </si>
   <si>
     <t>benefits_daily_6am</t>
   </si>
   <si>
     <t>Y</t>
+  </si>
+  <si>
+    <t>BatchEligibilityLoad</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>benefits_daily_8am</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>BatchDependentVerification</t>
+  </si>
+  <si>
+    <t>REPORT_TYPE=FULL</t>
+  </si>
+  <si>
+    <t>benefits_daily_930am</t>
+  </si>
+  <si>
+    <t>BatchLifeEventProcessor</t>
+  </si>
+  <si>
+    <t>benefits_daily_4pm</t>
+  </si>
+  <si>
+    <t>BatchCoverageChangeNotifier</t>
+  </si>
+  <si>
+    <t>NOTIFY=EMAIL,SMS</t>
+  </si>
+  <si>
+    <t>benefits_daily_515pm</t>
+  </si>
+  <si>
+    <t>BatchBeneficiaryUpdate</t>
+  </si>
+  <si>
+    <t>benefits_daily_9pm</t>
+  </si>
+  <si>
+    <t>BatchPremiumCalculation</t>
+  </si>
+  <si>
+    <t>CALC_MODE=STANDARD</t>
+  </si>
+  <si>
+    <t>benefits_daily_1030am</t>
+  </si>
+  <si>
+    <t>BatchHSAContributionPost</t>
+  </si>
+  <si>
+    <t>benefits_daily_0630pm</t>
+  </si>
+  <si>
+    <t>BatchWeeklyEnrollmentReport</t>
+  </si>
+  <si>
+    <t>FORMAT=PDF,RECIPIENT=hr-team@corp.com</t>
+  </si>
+  <si>
+    <t>benefits_weekly_friday_6am</t>
+  </si>
+  <si>
+    <t>BatchCobraEligibilityCheck</t>
+  </si>
+  <si>
+    <t>benefits_weekly_monday_6am</t>
+  </si>
+  <si>
+    <t>BatchDentalClaimsReconcile</t>
+  </si>
+  <si>
+    <t>PLAN_YEAR=2024</t>
+  </si>
+  <si>
+    <t>benefits_weekly_wednesday_6am</t>
+  </si>
+  <si>
+    <t>BatchVisionBenefitsAudit</t>
+  </si>
+  <si>
+    <t>benefits_weekly_thursday_9am</t>
+  </si>
+  <si>
+    <t>BatchWellnessIncentiveCalc</t>
+  </si>
+  <si>
+    <t>PROGRAM=WELLNESS2024</t>
+  </si>
+  <si>
+    <t>benefits_weekly_tuesday_6am</t>
+  </si>
+  <si>
+    <t>BatchFSABalanceReconcile</t>
+  </si>
+  <si>
+    <t>TAX_YEAR=2024</t>
+  </si>
+  <si>
+    <t>benefits_monthly_1st_day_6am</t>
+  </si>
+  <si>
+    <t>BatchHRAMonthlyStatement</t>
+  </si>
+  <si>
+    <t>benefits_monthly_3rd_day_6am</t>
+  </si>
+  <si>
+    <t>BatchOpenEnrollmentSummary</t>
+  </si>
+  <si>
+    <t>OE_YEAR=2024,FINALIZE=true</t>
+  </si>
+  <si>
+    <t>benefits_monthly_8th_day_6am</t>
+  </si>
+  <si>
+    <t>BatchDependentAuditReport</t>
+  </si>
+  <si>
+    <t>INCLUDE_INACTIVE=false</t>
+  </si>
+  <si>
+    <t>benefits_monthly_15th_day_6am</t>
+  </si>
+  <si>
+    <t>BatchBenefitsCostAnalysis</t>
+  </si>
+  <si>
+    <t>benefits_monthly_last_day_7pm</t>
+  </si>
+  <si>
+    <t>BatchQtrlyBenefitsSummary</t>
+  </si>
+  <si>
+    <t>QUARTER=Q2_2024</t>
+  </si>
+  <si>
+    <t>benefits_qtrly_1st_day</t>
+  </si>
+  <si>
+    <t>BatchACAEligibilityBuild</t>
+  </si>
+  <si>
+    <t>YEAR=2024,EMPLOYER_ID=EMP001</t>
+  </si>
+  <si>
+    <t>benefits_qtrly_9th_day</t>
+  </si>
+  <si>
+    <t>BatchOpenEnrollmentEligLoad</t>
+  </si>
+  <si>
+    <t>FILE=/data/elig/oe2024.csv</t>
+  </si>
+  <si>
+    <t>on_demand</t>
+  </si>
+  <si>
+    <t>BatchBenefitsIconExport</t>
+  </si>
+  <si>
+    <t>EXPORT_TYPE=FULL</t>
+  </si>
+  <si>
+    <t>benefits_icon_export_10am</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -49,13 +220,21 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9E1F2"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -70,8 +249,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -411,20 +591,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="36" customWidth="1"/>
+    <col min="2" max="2" width="40" customWidth="1"/>
+    <col min="3" max="3" width="42" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
@@ -440,6 +626,300 @@
       </c>
       <c r="D2" t="s">
         <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" t="s">
+        <v>29</v>
+      </c>
+      <c r="D10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>30</v>
+      </c>
+      <c r="B11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" t="s">
+        <v>31</v>
+      </c>
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>32</v>
+      </c>
+      <c r="B12" t="s">
+        <v>33</v>
+      </c>
+      <c r="C12" t="s">
+        <v>34</v>
+      </c>
+      <c r="D12" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" t="s">
+        <v>36</v>
+      </c>
+      <c r="D13" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>37</v>
+      </c>
+      <c r="B14" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14" t="s">
+        <v>39</v>
+      </c>
+      <c r="D14" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>40</v>
+      </c>
+      <c r="B15" t="s">
+        <v>41</v>
+      </c>
+      <c r="C15" t="s">
+        <v>42</v>
+      </c>
+      <c r="D15" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>43</v>
+      </c>
+      <c r="B16" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>45</v>
+      </c>
+      <c r="B17" t="s">
+        <v>46</v>
+      </c>
+      <c r="C17" t="s">
+        <v>47</v>
+      </c>
+      <c r="D17" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>48</v>
+      </c>
+      <c r="B18" t="s">
+        <v>49</v>
+      </c>
+      <c r="C18" t="s">
+        <v>50</v>
+      </c>
+      <c r="D18" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>51</v>
+      </c>
+      <c r="B19" t="s">
+        <v>9</v>
+      </c>
+      <c r="C19" t="s">
+        <v>52</v>
+      </c>
+      <c r="D19" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>53</v>
+      </c>
+      <c r="B20" t="s">
+        <v>54</v>
+      </c>
+      <c r="C20" t="s">
+        <v>55</v>
+      </c>
+      <c r="D20" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>56</v>
+      </c>
+      <c r="B21" t="s">
+        <v>57</v>
+      </c>
+      <c r="C21" t="s">
+        <v>58</v>
+      </c>
+      <c r="D21" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>59</v>
+      </c>
+      <c r="B22" t="s">
+        <v>60</v>
+      </c>
+      <c r="C22" t="s">
+        <v>61</v>
+      </c>
+      <c r="D22" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>62</v>
+      </c>
+      <c r="B23" t="s">
+        <v>63</v>
+      </c>
+      <c r="C23" t="s">
+        <v>64</v>
+      </c>
+      <c r="D23" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>